<commit_message>
Prepare chair review allocation updates
</commit_message>
<xml_diff>
--- a/outputs/bah_comment_collation/BAH_Draft_Review_Comment_Register.xlsx
+++ b/outputs/bah_comment_collation/BAH_Draft_Review_Comment_Register.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rbe110c64bcb942bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comment Register" sheetId="2" r:id="Rd16331fc83fb4bb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BAH Response" sheetId="3" r:id="R7fb599bb68af48cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Document Summary" sheetId="4" r:id="R27731da164a347b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2a34960cbf494c05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comment Register" sheetId="2" r:id="Rf815880eeed745dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BAH Response" sheetId="3" r:id="R6ce93034913b43e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Document Summary" sheetId="4" r:id="R079c43bd8ef14566"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1175,7 +1175,7 @@
         <x:v>PP-Configuration-Server-Agent-v2.0-draft-review-BAH.pdf</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="66" hidden="0" customHeight="1">
+    <x:row r="6" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A6" s="74" t="str">
         <x:v>BAH-005</x:v>
       </x:c>
@@ -1210,13 +1210,13 @@
         <x:v>Resolved</x:v>
       </x:c>
       <x:c r="L6" s="76" t="str">
-        <x:v>Accept with adaptation</x:v>
+        <x:v>Accept</x:v>
       </x:c>
       <x:c r="M6" s="76" t="str">
         <x:v>AppSW-iTC</x:v>
       </x:c>
       <x:c r="N6" s="76" t="str">
-        <x:v>Retained Applicable Components for component allocation. Feature Dependent is now explicitly a condition of applicability, not an alternative allocation that can narrow coverage.</x:v>
+        <x:v>Adopted the NDcPP distributed-TOE allocation vocabulary. The configuration now uses only All Components, At Least One Component, and Feature Dependent. A Feature Dependent SFR element is fulfilled where its feature is implemented; the ST maps every implementing component to its element. A separate claim condition records inclusion without narrowing component coverage.</x:v>
       </x:c>
       <x:c r="O6" s="76" t="str">
         <x:v>PP-Configuration-Server-Agent-v2.0-draft-review-BAH.pdf</x:v>
@@ -1257,13 +1257,13 @@
         <x:v>Resolved</x:v>
       </x:c>
       <x:c r="L7" s="76" t="str">
-        <x:v>Accept with adaptation</x:v>
+        <x:v>Accept</x:v>
       </x:c>
       <x:c r="M7" s="76" t="str">
         <x:v>AppSW-iTC</x:v>
       </x:c>
       <x:c r="N7" s="76" t="str">
-        <x:v>Clarified the two-stage model: a feature or selection determines whether an SFR is claimed; Applicable Components identifies every component with a concrete obligation once it is claimed.</x:v>
+        <x:v>Replaced Applicable Components with the NDcPP Feature Dependent allocation. The required element-level mapping, evaluation coverage, and evidence-reuse controls remain; Feature Dependent is not an additional optionality mechanism.</x:v>
       </x:c>
       <x:c r="O7" s="76" t="str">
         <x:v>PP-Configuration-Server-Agent-v2.0-draft-review-BAH.pdf</x:v>
@@ -1310,13 +1310,13 @@
         <x:v>AppSW-iTC</x:v>
       </x:c>
       <x:c r="N8" s="76" t="str">
-        <x:v>Reframed the allocation rationale around allocation category plus feature-dependent condition, retained network-stack coverage independent of locality, and limited non-network IPC documentation to architecture-level protection unless an SFR or EA needs more detail.</x:v>
+        <x:v>Aligned the allocation rationale to the NDcPP All Components, At Least One Component, and Feature Dependent terminology while retaining the independent loopback and non-network IPC resolution. Non-network IPC identification and protection are addressed by the objective FPT_IPC_EXT.1 rather than by a mandatory allocation rule.</x:v>
       </x:c>
       <x:c r="O8" s="76" t="str">
         <x:v>PP-Configuration-Server-Agent-v2.0-draft-review-BAH.pdf</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="66" hidden="0" customHeight="1">
+    <x:row r="9" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A9" s="74" t="str">
         <x:v>BAH-008</x:v>
       </x:c>
@@ -1351,13 +1351,13 @@
         <x:v>Resolved</x:v>
       </x:c>
       <x:c r="L9" s="76" t="str">
-        <x:v>Accept with adaptation</x:v>
+        <x:v>Accept</x:v>
       </x:c>
       <x:c r="M9" s="76" t="str">
         <x:v>AppSW-iTC</x:v>
       </x:c>
       <x:c r="N9" s="76" t="str">
-        <x:v>Specified element-level allocation. Components need satisfy only the SFR elements they implement, while the evaluation evidence jointly covers every allocated element and cannot be satisfied by a representative component without demonstrated equivalence.</x:v>
+        <x:v>Adopted Feature Dependent and explicitly maps multi-element SFRs at the element level. Each component satisfies only the elements it implements, and the mapped elements collectively satisfy the TOE-level SFR. The FCO_CPC example maps enablement, registration, and disablement separately; evaluation evidence jointly covers every mapped element, without relying on a Server test to prove a distinct Agent path absent demonstrated equivalent implementation, configuration, and execution context.</x:v>
       </x:c>
       <x:c r="O9" s="76" t="str">
         <x:v>PP-Configuration-Server-Agent-v2.0-draft-review-BAH.pdf</x:v>
@@ -3190,13 +3190,13 @@
         <x:v>AppSW-iTC</x:v>
       </x:c>
       <x:c r="N48" s="76" t="str">
-        <x:v>Retained the base cPP obligation to identify non-network IPC and clarified in the Server-Agent configuration that the description is limited to the mechanism and architecture-level protection relied upon. Detailed implementation or configuration information is required only when an SFR or EA requires it.</x:v>
+        <x:v>Moved the non-network IPC identification and protection rationale from the mandatory FTP_DIT_EXT.1 application note to the objective FPT_IPC_EXT.1. The Server-Agent configuration directs non-network IPC protection to that objective; its Evaluation Activities identify the mechanism and architecture-level protection relied upon.</x:v>
       </x:c>
       <x:c r="O48" s="76" t="str">
         <x:v>cPP-Application-Software-v2.0-draft-review - BAH.pdf</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="79.19999694824219" hidden="0" customHeight="1">
+    <x:row r="49" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A49" s="74" t="str">
         <x:v>BAH-048</x:v>
       </x:c>
@@ -3237,7 +3237,7 @@
         <x:v>AppSW-iTC</x:v>
       </x:c>
       <x:c r="N49" s="76" t="str">
-        <x:v>Confirmed the intended outcome: a database service reached through a network stack, including loopback, is a transmitted-data endpoint. The ST identifies it as a TOE Component Instance or selected trusted IT product; in-process calls and direct local storage remain outside FTP_DIT_EXT.1. A loopback path is explicitly exercised where present.</x:v>
+        <x:v>Aligned the cPP with the confirmed NIAP AppSW v2.0 scope: a database service reached only through the platform loopback interface is not an FTP_DIT_EXT.1 transmitted-data endpoint and is not separately tested. This boundary does not assume that local users, processes, or localhost traffic are trusted; it only does not create an evaluated trusted-channel claim in this cPP version. In-scope network-mediated communications to a trusted IT product or TOE Component Instance remain covered. In-process calls and direct local storage remain outside FTP_DIT_EXT.1; non-network IPC is addressed by the FPT_IPC_EXT.1 objective.</x:v>
       </x:c>
       <x:c r="O49" s="76" t="str">
         <x:v>cPP-Application-Software-v2.0-draft-review - BAH.pdf</x:v>
@@ -3305,7 +3305,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4045f6a377aa4dab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74d819fa0e3a4419"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3453,13 +3453,13 @@
         <x:v>Distributed TOE allocation, IPC, and loopback scope</x:v>
       </x:c>
       <x:c r="D9" s="76" t="str">
-        <x:v>Accept with adaptation</x:v>
+        <x:v>Accept</x:v>
       </x:c>
       <x:c r="E9" s="76" t="str">
-        <x:v>Retained Applicable Components for component allocation. Feature Dependent is now explicitly a condition of applicability, not an alternative allocation that can narrow coverage.</x:v>
+        <x:v>Adopted the NDcPP distributed-TOE allocation vocabulary. The configuration now uses only All Components, At Least One Component, and Feature Dependent. A Feature Dependent SFR element is fulfilled where its feature is implemented; the ST maps every implementing component to its element. A separate claim condition records inclusion without narrowing component coverage.</x:v>
       </x:c>
       <x:c r="F9" s="76" t="str">
-        <x:v>Server-Agent configuration, allocation definitions and worked example</x:v>
+        <x:v>Base cPP and Server-Agent configuration, allocation rationale, required ST mapping, and worked example</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="72" customHeight="1">
@@ -3473,13 +3473,13 @@
         <x:v>Distributed TOE allocation, IPC, and loopback scope</x:v>
       </x:c>
       <x:c r="D10" s="76" t="str">
-        <x:v>Accept with adaptation</x:v>
+        <x:v>Accept</x:v>
       </x:c>
       <x:c r="E10" s="76" t="str">
-        <x:v>Clarified the two-stage model: a feature or selection determines whether an SFR is claimed; Applicable Components identifies every component with a concrete obligation once it is claimed.</x:v>
+        <x:v>Replaced Applicable Components with the NDcPP Feature Dependent allocation. The required element-level mapping, evaluation coverage, and evidence-reuse controls remain; Feature Dependent is not an additional optionality mechanism.</x:v>
       </x:c>
       <x:c r="F10" s="76" t="str">
-        <x:v>Server-Agent configuration, allocation definitions and worked example</x:v>
+        <x:v>Base cPP and Server-Agent configuration, allocation rationale, ST mapping, and worked example</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="72" customHeight="1">
@@ -3496,10 +3496,10 @@
         <x:v>Accept with adaptation</x:v>
       </x:c>
       <x:c r="E11" s="76" t="str">
-        <x:v>Reframed the allocation rationale around allocation category plus feature-dependent condition, retained network-stack coverage independent of locality, and limited non-network IPC documentation to architecture-level protection unless an SFR or EA needs more detail.</x:v>
+        <x:v>Aligned the allocation rationale to the NDcPP All Components, At Least One Component, and Feature Dependent terminology while retaining the independent loopback and non-network IPC resolution. Non-network IPC identification and protection are addressed by the objective FPT_IPC_EXT.1 rather than by a mandatory allocation rule.</x:v>
       </x:c>
       <x:c r="F11" s="76" t="str">
-        <x:v>Server-Agent configuration, distributed TOE rationale</x:v>
+        <x:v>Server-Agent configuration and base cPP, distributed TOE rationale</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="72" customHeight="1">
@@ -3513,13 +3513,13 @@
         <x:v>Distributed TOE allocation, IPC, and loopback scope</x:v>
       </x:c>
       <x:c r="D12" s="76" t="str">
-        <x:v>Accept with adaptation</x:v>
+        <x:v>Accept</x:v>
       </x:c>
       <x:c r="E12" s="76" t="str">
-        <x:v>Specified element-level allocation. Components need satisfy only the SFR elements they implement, while the evaluation evidence jointly covers every allocated element and cannot be satisfied by a representative component without demonstrated equivalence.</x:v>
+        <x:v>Adopted Feature Dependent and explicitly maps multi-element SFRs at the element level. Each component satisfies only the elements it implements, and the mapped elements collectively satisfy the TOE-level SFR. The FCO_CPC example maps enablement, registration, and disablement separately; evaluation evidence jointly covers every mapped element, without relying on a Server test to prove a distinct Agent path absent demonstrated equivalent implementation, configuration, and execution context.</x:v>
       </x:c>
       <x:c r="F12" s="76" t="str">
-        <x:v>Server-Agent configuration, allocation rule and FPT_TUD_EXT.2 example</x:v>
+        <x:v>Base cPP and Server-Agent configuration, allocation rationale, FCO_CPC mapping, and FPT_TUD_EXT.2 example</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="72" customHeight="1">
@@ -4296,10 +4296,10 @@
         <x:v>Accept with adaptation</x:v>
       </x:c>
       <x:c r="E51" s="76" t="str">
-        <x:v>Retained the base cPP obligation to identify non-network IPC and clarified in the Server-Agent configuration that the description is limited to the mechanism and architecture-level protection relied upon. Detailed implementation or configuration information is required only when an SFR or EA requires it.</x:v>
+        <x:v>Moved the non-network IPC identification and protection rationale from the mandatory FTP_DIT_EXT.1 application note to the objective FPT_IPC_EXT.1. The Server-Agent configuration directs non-network IPC protection to that objective; its Evaluation Activities identify the mechanism and architecture-level protection relied upon.</x:v>
       </x:c>
       <x:c r="F51" s="76" t="str">
-        <x:v>Base cPP and Server-Agent configuration, distributed-TOE IPC guidance</x:v>
+        <x:v>Base cPP FPT_IPC_EXT.1 and Server-Agent configuration, distributed-TOE IPC guidance</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="72" customHeight="1">
@@ -4316,7 +4316,7 @@
         <x:v>Clarify with reviewer</x:v>
       </x:c>
       <x:c r="E52" s="76" t="str">
-        <x:v>Confirmed the intended outcome: a database service reached through a network stack, including loopback, is a transmitted-data endpoint. The ST identifies it as a TOE Component Instance or selected trusted IT product; in-process calls and direct local storage remain outside FTP_DIT_EXT.1. A loopback path is explicitly exercised where present.</x:v>
+        <x:v>Aligned the cPP with the confirmed NIAP AppSW v2.0 scope: a database service reached only through the platform loopback interface is not an FTP_DIT_EXT.1 transmitted-data endpoint and is not separately tested. This boundary does not assume that local users, processes, or localhost traffic are trusted; it only does not create an evaluated trusted-channel claim in this cPP version. In-scope network-mediated communications to a trusted IT product or TOE Component Instance remain covered. In-process calls and direct local storage remain outside FTP_DIT_EXT.1; non-network IPC is addressed by the FPT_IPC_EXT.1 objective.</x:v>
       </x:c>
       <x:c r="F52" s="76" t="str">
         <x:v>Base cPP, FTP_DIT_EXT.1 target selection and EA</x:v>
@@ -4353,7 +4353,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5645371b89241e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb0e4beb1de54c78"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>